<commit_message>
function to clean it up a bit
</commit_message>
<xml_diff>
--- a/OutputData/StandardErrorCalculations/errorSummarizedDFs2025.xlsx
+++ b/OutputData/StandardErrorCalculations/errorSummarizedDFs2025.xlsx
@@ -7,9 +7,9 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="trimbleM3SummarizedFinal" sheetId="1" r:id="rId1"/>
-    <sheet name="trimbleM4SummarizedFinal" sheetId="2" r:id="rId2"/>
-    <sheet name="trimbleHPRSummarizedFinal" sheetId="3" r:id="rId3"/>
+    <sheet name="trimblevsM3SummarizedFinal" sheetId="1" r:id="rId1"/>
+    <sheet name="trimblevsM4SummarizedFinal" sheetId="2" r:id="rId2"/>
+    <sheet name="trimblevsHPRSummarizedFinal" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -359,7 +359,7 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>antennaTypeM3</t>
+          <t>antennaType</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -606,7 +606,7 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>antennaTypeM4</t>
+          <t>antennaType</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -748,7 +748,7 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>antennaTypeHPR</t>
+          <t>antennaType</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">

</xml_diff>